<commit_message>
INVENTORI IMPORT AND LPB EXPORT
</commit_message>
<xml_diff>
--- a/public/assets/import/IMPORT_EXCEL_MASTER_BJ.xlsx
+++ b/public/assets/import/IMPORT_EXCEL_MASTER_BJ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ardhi\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38A2FA37-6497-4387-84E3-BC79113A32F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60B8D444-90C8-4392-B9D9-8D676E06DCF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -48,16 +48,16 @@
     <t>KODE SATUAN (*)</t>
   </si>
   <si>
-    <t>BJ - 1111</t>
-  </si>
-  <si>
-    <t>BJ - 1115</t>
-  </si>
-  <si>
     <t>DG UDANG</t>
   </si>
   <si>
     <t>DG KEPITING</t>
+  </si>
+  <si>
+    <t>BJ-1111</t>
+  </si>
+  <si>
+    <t>BJ-1115</t>
   </si>
 </sst>
 </file>
@@ -430,20 +430,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="24.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.3984375" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
-    <col min="3" max="3" width="33.140625" customWidth="1"/>
-    <col min="4" max="4" width="35.28515625" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" customWidth="1"/>
-    <col min="6" max="6" width="26.85546875" customWidth="1"/>
-    <col min="7" max="7" width="31.28515625" customWidth="1"/>
-    <col min="8" max="8" width="25.7109375" customWidth="1"/>
-    <col min="9" max="9" width="29.28515625" customWidth="1"/>
+    <col min="3" max="3" width="33.1328125" customWidth="1"/>
+    <col min="4" max="4" width="35.265625" customWidth="1"/>
+    <col min="5" max="5" width="17.59765625" customWidth="1"/>
+    <col min="6" max="6" width="26.86328125" customWidth="1"/>
+    <col min="7" max="7" width="31.265625" customWidth="1"/>
+    <col min="8" max="8" width="25.73046875" customWidth="1"/>
+    <col min="9" max="9" width="29.265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="2" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="3" t="s">
         <v>2</v>
       </c>
@@ -464,15 +464,15 @@
       <c r="H1" s="4"/>
       <c r="I1" s="5"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="D2" s="1">
         <v>314</v>
@@ -485,15 +485,15 @@
       <c r="H2" s="1"/>
       <c r="I2" s="6"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="D3" s="1">
         <v>276</v>
@@ -506,15 +506,15 @@
       <c r="H3" s="1"/>
       <c r="I3" s="6"/>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="D4" s="1">
         <v>316</v>
@@ -527,15 +527,15 @@
       <c r="H4" s="1"/>
       <c r="I4" s="6"/>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>9</v>
       </c>
       <c r="D5" s="1">
         <v>288</v>
@@ -548,15 +548,15 @@
       <c r="H5" s="1"/>
       <c r="I5" s="6"/>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>8</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>10</v>
       </c>
       <c r="D6" s="1">
         <v>276</v>
@@ -569,7 +569,7 @@
       <c r="H6" s="1"/>
       <c r="I6" s="6"/>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="1"/>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -580,7 +580,7 @@
       <c r="H7" s="1"/>
       <c r="I7" s="6"/>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -591,7 +591,7 @@
       <c r="H8" s="1"/>
       <c r="I8" s="6"/>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -602,7 +602,7 @@
       <c r="H9" s="1"/>
       <c r="I9" s="6"/>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
@@ -613,7 +613,7 @@
       <c r="H10" s="1"/>
       <c r="I10" s="6"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
@@ -624,7 +624,7 @@
       <c r="H11" s="1"/>
       <c r="I11" s="6"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
@@ -635,7 +635,7 @@
       <c r="H12" s="1"/>
       <c r="I12" s="6"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
@@ -646,7 +646,7 @@
       <c r="H13" s="1"/>
       <c r="I13" s="6"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>

</xml_diff>